<commit_message>
merging enzyme complex was counting molarmasses and lenghts double due to duplicates entries. Dropping duplicates and looping over direction resolves issue
</commit_message>
<xml_diff>
--- a/tests/data/enzyme_complexes_to_merge_info.xlsx
+++ b/tests/data/enzyme_complexes_to_merge_info.xlsx
@@ -5,11 +5,11 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="f_b_multiple_complexes_atps" sheetId="1" state="visible" r:id="rId2"/>
-    <sheet name="mixed_and_or_gpr_different_comp" sheetId="2" state="visible" r:id="rId3"/>
+    <sheet name="mixed_and_or_gpr" sheetId="2" state="visible" r:id="rId3"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="349" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="58">
   <si>
     <t xml:space="preserve">rxn_id</t>
   </si>
@@ -176,16 +176,25 @@
     <t xml:space="preserve">ANS</t>
   </si>
   <si>
-    <t xml:space="preserve">cg3361 or (cg3360 and cg3359) or (cg3361 and cg3359)'</t>
+    <t xml:space="preserve">cg3361 or (cg3360 and cg3359) or (cg3361 and cg3359)</t>
   </si>
   <si>
     <t xml:space="preserve">Enzyme_cg3361</t>
   </si>
   <si>
+    <t xml:space="preserve">cg3361</t>
+  </si>
+  <si>
     <t xml:space="preserve">Enzyme_cg3360</t>
   </si>
   <si>
+    <t xml:space="preserve">cg3360</t>
+  </si>
+  <si>
     <t xml:space="preserve">Enzyme_cg3359</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cg3359</t>
   </si>
 </sst>
 </file>
@@ -277,7 +286,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -287,6 +296,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -312,7 +325,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:O35"/>
-  <sheetFormatPr defaultColWidth="8.6875" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.72265625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1024" min="1024" style="0" width="11.52"/>
   </cols>
@@ -1658,7 +1671,7 @@
       <c r="D32" s="0" t="s">
         <v>18</v>
       </c>
-      <c r="E32" s="0" t="b">
+      <c r="E32" s="2" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -1703,7 +1716,7 @@
       <c r="D33" s="0" t="s">
         <v>18</v>
       </c>
-      <c r="E33" s="0" t="b">
+      <c r="E33" s="2" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -1745,7 +1758,7 @@
       <c r="D34" s="0" t="s">
         <v>18</v>
       </c>
-      <c r="E34" s="0" t="b">
+      <c r="E34" s="2" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -1787,7 +1800,7 @@
       <c r="D35" s="0" t="s">
         <v>18</v>
       </c>
-      <c r="E35" s="0" t="b">
+      <c r="E35" s="2" t="b">
         <f aca="false">TRUE()</f>
         <v>1</v>
       </c>
@@ -1833,7 +1846,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H4"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -1843,91 +1856,100 @@
         <v>3</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="H1" s="1" t="s">
         <v>14</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
         <v>50</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="C2" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="E2" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="F2" s="3" t="n">
+      <c r="D2" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" s="4" t="n">
         <v>39959.4825</v>
       </c>
-      <c r="G2" s="3" t="n">
+      <c r="F2" s="4" t="n">
         <v>0.0449</v>
       </c>
+      <c r="G2" s="0" t="s">
+        <v>23</v>
+      </c>
       <c r="H2" s="0" t="s">
-        <v>23</v>
+        <v>53</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
         <v>50</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="D3" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="E3" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="F3" s="3" t="n">
+      <c r="C3" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D3" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" s="4" t="n">
         <v>39959.4825</v>
       </c>
-      <c r="G3" s="3" t="n">
+      <c r="F3" s="4" t="n">
         <v>0.0449</v>
       </c>
+      <c r="G3" s="0" t="s">
+        <v>23</v>
+      </c>
       <c r="H3" s="0" t="s">
-        <v>23</v>
+        <v>55</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
         <v>50</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="D4" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="E4" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="F4" s="3" t="n">
+      <c r="C4" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="D4" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="4" t="n">
         <v>39959.4825</v>
       </c>
-      <c r="G4" s="3" t="n">
+      <c r="F4" s="4" t="n">
         <v>0.0449</v>
       </c>
+      <c r="G4" s="0" t="s">
+        <v>23</v>
+      </c>
       <c r="H4" s="0" t="s">
-        <v>23</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>